<commit_message>
inorder traversal + vktest
</commit_message>
<xml_diff>
--- a/lab7/lab7.xlsx
+++ b/lab7/lab7.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\AlgoC++\code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\AlgoC++\lab7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17DA45D-A39C-424F-8F3A-FBBBD3150F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB89F303-C9CA-4F9A-BE5F-D25890DFFFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2C66FF05-2C4F-446F-8D54-368B8A175AF5}"/>
   </bookViews>
@@ -3262,6 +3262,9 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>Декартово</c:v>
+          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -3407,6 +3410,9 @@
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>АВЛ</c:v>
+          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:schemeClr val="accent2"/>
@@ -3776,6 +3782,42 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="39000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>

</xml_diff>